<commit_message>
Criar documentação do análise da etapa 4 da release 2 do projeto Gestão de Movimentações
</commit_message>
<xml_diff>
--- a/docs/aplicacoes/gestao-movimentacoes/release-2/etapa-4/anexos/Comarcas a corrigir SIGEP.xlsx
+++ b/docs/aplicacoes/gestao-movimentacoes/release-2/etapa-4/anexos/Comarcas a corrigir SIGEP.xlsx
@@ -5,25 +5,22 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felipe.stella\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Analises\docs\aplicacoes\gestao-movimentacoes\release-2\etapa-4\anexos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3B3458-FEE2-4DD7-AB39-583A207FF930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B370C88F-B10F-41F1-8E27-AB5EA563CA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{033D172E-D4BC-4874-852D-DADC2315DC54}"/>
   </bookViews>
   <sheets>
     <sheet name="Comarcas a corrigir SIGEP" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="144">
-  <si>
-    <t>Comarca SIGEP</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="128">
   <si>
     <t>Marcio Cristiano de Castro Scotti</t>
   </si>
@@ -64,9 +61,6 @@
     <t>Bianca Hagemann Behling Alves</t>
   </si>
   <si>
-    <t>Comarca de Santa Maria</t>
-  </si>
-  <si>
     <t>Comarca de Frederico Westphalen</t>
   </si>
   <si>
@@ -85,9 +79,6 @@
     <t>Pedro Henrique Cunha Martini</t>
   </si>
   <si>
-    <t>Comarca de Cachoeirinha</t>
-  </si>
-  <si>
     <t>Comarca de São Sepé</t>
   </si>
   <si>
@@ -118,9 +109,6 @@
     <t>Felipe Hanauer Bertotto</t>
   </si>
   <si>
-    <t>Comarca de Novo Hamburgo</t>
-  </si>
-  <si>
     <t>Comarca de Espumoso</t>
   </si>
   <si>
@@ -169,9 +157,6 @@
     <t>Joao Flavio Evangelista</t>
   </si>
   <si>
-    <t>Comarca de Igrejinha</t>
-  </si>
-  <si>
     <t>Maiara Ferrao</t>
   </si>
   <si>
@@ -211,9 +196,6 @@
     <t>Sara Simoni Kahl</t>
   </si>
   <si>
-    <t>Comarca de São Leopoldo</t>
-  </si>
-  <si>
     <t>Luana Bianca Freitas dos Santos</t>
   </si>
   <si>
@@ -229,9 +211,6 @@
     <t>Luciano Sesti Destro</t>
   </si>
   <si>
-    <t>Comarca de Marau</t>
-  </si>
-  <si>
     <t>Bianca Roloff Serafim</t>
   </si>
   <si>
@@ -271,21 +250,12 @@
     <t>Carolina Dutra de Deus</t>
   </si>
   <si>
-    <t>Comarca de Capão da Canoa</t>
-  </si>
-  <si>
     <t>Ana Maria Gauterio Tavares</t>
   </si>
   <si>
-    <t>Comarca de Ivoti</t>
-  </si>
-  <si>
     <t>Jaques Douglas Paim</t>
   </si>
   <si>
-    <t>Comarca de Camaquã</t>
-  </si>
-  <si>
     <t>Caio Sergio Siqueira de Mello</t>
   </si>
   <si>
@@ -304,9 +274,6 @@
     <t>Patrícia Mendel Soares</t>
   </si>
   <si>
-    <t>Comarca de Crissiumal</t>
-  </si>
-  <si>
     <t>Comarca de Santa Rosa</t>
   </si>
   <si>
@@ -340,21 +307,12 @@
     <t>Roberto Franz Blödorn</t>
   </si>
   <si>
-    <t>Comarca de Parobé</t>
-  </si>
-  <si>
     <t>Joana Arenhart</t>
   </si>
   <si>
-    <t>Comarca de Arroio do Meio</t>
-  </si>
-  <si>
     <t>Wendell Larruscain da Silva</t>
   </si>
   <si>
-    <t>Comarca de Esteio</t>
-  </si>
-  <si>
     <t>Lucia Giacobo Pinho Mendes</t>
   </si>
   <si>
@@ -364,9 +322,6 @@
     <t>Daniela Cristina Menin</t>
   </si>
   <si>
-    <t>Comarca de Nonoai</t>
-  </si>
-  <si>
     <t>Comarca de Erechim</t>
   </si>
   <si>
@@ -376,9 +331,6 @@
     <t>Everton Ferri</t>
   </si>
   <si>
-    <t>Comarca de Bento Gonçalves</t>
-  </si>
-  <si>
     <t>Comarca de Santo Ângelo</t>
   </si>
   <si>
@@ -451,7 +403,7 @@
     <t>DtInicioAtividades</t>
   </si>
   <si>
-    <t>Testar alinhamento comarca origem</t>
+    <t>Ricardo Elias Paiva Moreira</t>
   </si>
 </sst>
 </file>
@@ -935,9 +887,19 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1313,38 +1275,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63C13787-6330-4CC6-AE87-CABAE1AA2419}">
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="39.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.33203125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>3414213</v>
       </c>
@@ -1352,16 +1311,20 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E2" s="2">
+        <v>44629</v>
+      </c>
+      <c r="F2" s="3" t="str">
+        <f ca="1">DATEDIF(E2,TODAY(),"y")&amp;" anos, "&amp;DATEDIF(E2,TODAY(),"ym")&amp;" meses e "&amp;DATEDIF(E2,TODAY(),"md")&amp;" dias"</f>
+        <v>4 anos, 3 meses e 10 dias</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>4235266</v>
       </c>
@@ -1369,19 +1332,20 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E3" s="2">
+        <v>44629</v>
+      </c>
+      <c r="F3" s="3" t="str">
+        <f t="shared" ref="F3:F66" ca="1" si="0">DATEDIF(E3,TODAY(),"y")&amp;" anos, "&amp;DATEDIF(E3,TODAY(),"ym")&amp;" meses e "&amp;DATEDIF(E3,TODAY(),"md")&amp;" dias"</f>
+        <v>4 anos, 3 meses e 10 dias</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4573110</v>
       </c>
@@ -1389,16 +1353,20 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
         <v>6</v>
       </c>
-      <c r="D4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E4" s="2">
+        <v>44629</v>
+      </c>
+      <c r="F4" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>4 anos, 3 meses e 10 dias</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4456815</v>
       </c>
@@ -1406,16 +1374,20 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" t="s">
         <v>2</v>
       </c>
-      <c r="E5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E5" s="2">
+        <v>44637</v>
+      </c>
+      <c r="F5" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>4 anos, 3 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4242033</v>
       </c>
@@ -1423,16 +1395,20 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
         <v>9</v>
       </c>
-      <c r="D6" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E6" s="2">
+        <v>44748</v>
+      </c>
+      <c r="F6" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 11 meses e 13 dias</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>3052281</v>
       </c>
@@ -1440,16 +1416,20 @@
         <v>3</v>
       </c>
       <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s">
         <v>11</v>
       </c>
-      <c r="D7" t="s">
-        <v>2</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E7" s="2">
+        <v>44764</v>
+      </c>
+      <c r="F7" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 28 dias</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>4644719</v>
       </c>
@@ -1457,16 +1437,20 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
         <v>13</v>
       </c>
-      <c r="D8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E8" s="2">
+        <v>44764</v>
+      </c>
+      <c r="F8" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 28 dias</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>4804821</v>
       </c>
@@ -1474,16 +1458,20 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>5</v>
-      </c>
-      <c r="E9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="E9" s="2">
+        <v>44764</v>
+      </c>
+      <c r="F9" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 28 dias</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>4804996</v>
       </c>
@@ -1491,16 +1479,20 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="E10" s="2">
+        <v>44767</v>
+      </c>
+      <c r="F10" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 25 dias</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>3883540</v>
       </c>
@@ -1508,16 +1500,20 @@
         <v>3</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+      <c r="E11" s="2">
+        <v>44768</v>
+      </c>
+      <c r="F11" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>4698509</v>
       </c>
@@ -1525,16 +1521,20 @@
         <v>3</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="E12" s="2">
+        <v>44777</v>
+      </c>
+      <c r="F12" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 15 dias</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>4551664</v>
       </c>
@@ -1542,16 +1542,20 @@
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>5</v>
-      </c>
-      <c r="E13" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+      <c r="E13" s="2">
+        <v>44784</v>
+      </c>
+      <c r="F13" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 8 dias</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>4380177</v>
       </c>
@@ -1559,16 +1563,20 @@
         <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D14" t="s">
-        <v>5</v>
-      </c>
-      <c r="E14" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="E14" s="2">
+        <v>44785</v>
+      </c>
+      <c r="F14" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 7 dias</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>4804678</v>
       </c>
@@ -1576,16 +1584,20 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s">
-        <v>5</v>
-      </c>
-      <c r="E15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="E15" s="2">
+        <v>44785</v>
+      </c>
+      <c r="F15" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 7 dias</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>4812298</v>
       </c>
@@ -1593,16 +1605,20 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="E16" s="2">
+        <v>44790</v>
+      </c>
+      <c r="F16" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>4812450</v>
       </c>
@@ -1610,16 +1626,20 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D17" t="s">
-        <v>32</v>
-      </c>
-      <c r="E17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="E17" s="2">
+        <v>44790</v>
+      </c>
+      <c r="F17" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 10 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>4820274</v>
       </c>
@@ -1627,16 +1647,20 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D18" t="s">
-        <v>5</v>
-      </c>
-      <c r="E18" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+      <c r="E18" s="2">
+        <v>44799</v>
+      </c>
+      <c r="F18" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 9 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3401138</v>
       </c>
@@ -1644,16 +1668,20 @@
         <v>2</v>
       </c>
       <c r="C19" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D19" t="s">
-        <v>2</v>
-      </c>
-      <c r="E19" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+      <c r="E19" s="2">
+        <v>44812</v>
+      </c>
+      <c r="F19" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 9 meses e 11 dias</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>4486897</v>
       </c>
@@ -1661,16 +1689,20 @@
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D20" t="s">
-        <v>2</v>
-      </c>
-      <c r="E20" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E20" s="2">
+        <v>44812</v>
+      </c>
+      <c r="F20" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 9 meses e 11 dias</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>4213572</v>
       </c>
@@ -1678,16 +1710,20 @@
         <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D21" t="s">
-        <v>5</v>
-      </c>
-      <c r="E21" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+      <c r="E21" s="2">
+        <v>44813</v>
+      </c>
+      <c r="F21" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 9 meses e 10 dias</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>4457870</v>
       </c>
@@ -1695,16 +1731,20 @@
         <v>3</v>
       </c>
       <c r="C22" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D22" t="s">
-        <v>5</v>
-      </c>
-      <c r="E22" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="E22" s="2">
+        <v>44813</v>
+      </c>
+      <c r="F22" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 9 meses e 10 dias</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>4495535</v>
       </c>
@@ -1712,16 +1752,20 @@
         <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D23" t="s">
-        <v>2</v>
-      </c>
-      <c r="E23" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E23" s="2">
+        <v>44882</v>
+      </c>
+      <c r="F23" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 7 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>3880958</v>
       </c>
@@ -1729,16 +1773,20 @@
         <v>3</v>
       </c>
       <c r="C24" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D24" t="s">
-        <v>2</v>
-      </c>
-      <c r="E24" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E24" s="2">
+        <v>44883</v>
+      </c>
+      <c r="F24" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 7 meses e 1 dias</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>3862020</v>
       </c>
@@ -1746,16 +1794,20 @@
         <v>2</v>
       </c>
       <c r="C25" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D25" t="s">
-        <v>2</v>
-      </c>
-      <c r="E25" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E25" s="2">
+        <v>44887</v>
+      </c>
+      <c r="F25" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 6 meses e 28 dias</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>4276469</v>
       </c>
@@ -1763,16 +1815,20 @@
         <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>2</v>
-      </c>
-      <c r="E26" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E26" s="2">
+        <v>44887</v>
+      </c>
+      <c r="F26" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 6 meses e 28 dias</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>3406008</v>
       </c>
@@ -1780,16 +1836,20 @@
         <v>3</v>
       </c>
       <c r="C27" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D27" t="s">
-        <v>2</v>
-      </c>
-      <c r="E27" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E27" s="2">
+        <v>44888</v>
+      </c>
+      <c r="F27" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 6 meses e 27 dias</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>4201515</v>
       </c>
@@ -1797,16 +1857,20 @@
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D28" t="s">
-        <v>49</v>
-      </c>
-      <c r="E28" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E28" s="2">
+        <v>44894</v>
+      </c>
+      <c r="F28" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 6 meses e 21 dias</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>4282779</v>
       </c>
@@ -1814,16 +1878,20 @@
         <v>2</v>
       </c>
       <c r="C29" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D29" t="s">
-        <v>7</v>
-      </c>
-      <c r="E29" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E29" s="2">
+        <v>44894</v>
+      </c>
+      <c r="F29" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 6 meses e 21 dias</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>4595254</v>
       </c>
@@ -1831,16 +1899,20 @@
         <v>3</v>
       </c>
       <c r="C30" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D30" t="s">
-        <v>52</v>
-      </c>
-      <c r="E30" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E30" s="2">
+        <v>44894</v>
+      </c>
+      <c r="F30" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 6 meses e 21 dias</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>3452476</v>
       </c>
@@ -1848,16 +1920,20 @@
         <v>3</v>
       </c>
       <c r="C31" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D31" t="s">
-        <v>2</v>
-      </c>
-      <c r="E31" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E31" s="2">
+        <v>44900</v>
+      </c>
+      <c r="F31" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 6 meses e 14 dias</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>3748960</v>
       </c>
@@ -1865,16 +1941,20 @@
         <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D32" t="s">
-        <v>52</v>
-      </c>
-      <c r="E32" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E32" s="2">
+        <v>44900</v>
+      </c>
+      <c r="F32" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 6 meses e 14 dias</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>4557107</v>
       </c>
@@ -1882,16 +1962,20 @@
         <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D33" t="s">
-        <v>2</v>
-      </c>
-      <c r="E33" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="E33" s="2">
+        <v>44964</v>
+      </c>
+      <c r="F33" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 4 meses e 12 dias</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>3418243</v>
       </c>
@@ -1899,16 +1983,20 @@
         <v>3</v>
       </c>
       <c r="C34" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D34" t="s">
-        <v>2</v>
-      </c>
-      <c r="E34" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E34" s="2">
+        <v>44979</v>
+      </c>
+      <c r="F34" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 3 meses e 28 dias</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>3778819</v>
       </c>
@@ -1916,16 +2004,20 @@
         <v>3</v>
       </c>
       <c r="C35" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D35" t="s">
-        <v>2</v>
-      </c>
-      <c r="E35" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E35" s="2">
+        <v>44985</v>
+      </c>
+      <c r="F35" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 3 meses e 22 dias</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>4376749</v>
       </c>
@@ -1933,16 +2025,20 @@
         <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D36" t="s">
-        <v>19</v>
-      </c>
-      <c r="E36" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+        <v>54</v>
+      </c>
+      <c r="E36" s="2">
+        <v>44998</v>
+      </c>
+      <c r="F36" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>3 anos, 3 meses e 6 dias</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>4488741</v>
       </c>
@@ -1950,16 +2046,20 @@
         <v>2</v>
       </c>
       <c r="C37" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D37" t="s">
-        <v>2</v>
-      </c>
-      <c r="E37" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E37" s="2">
+        <v>45111</v>
+      </c>
+      <c r="F37" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 11 meses e 15 dias</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>4199286</v>
       </c>
@@ -1967,16 +2067,20 @@
         <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D38" t="s">
-        <v>52</v>
-      </c>
-      <c r="E38" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E38" s="2">
+        <v>45181</v>
+      </c>
+      <c r="F38" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 9 meses e 7 dias</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>4200454</v>
       </c>
@@ -1984,16 +2088,20 @@
         <v>2</v>
       </c>
       <c r="C39" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D39" t="s">
-        <v>63</v>
-      </c>
-      <c r="E39" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E39" s="2">
+        <v>45181</v>
+      </c>
+      <c r="F39" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 9 meses e 7 dias</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>4236530</v>
       </c>
@@ -2001,16 +2109,20 @@
         <v>2</v>
       </c>
       <c r="C40" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D40" t="s">
-        <v>32</v>
-      </c>
-      <c r="E40" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E40" s="2">
+        <v>45182</v>
+      </c>
+      <c r="F40" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 9 meses e 6 dias</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>3389545</v>
       </c>
@@ -2018,16 +2130,20 @@
         <v>2</v>
       </c>
       <c r="C41" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D41" t="s">
-        <v>2</v>
-      </c>
-      <c r="E41" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E41" s="2">
+        <v>45202</v>
+      </c>
+      <c r="F41" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>3664295</v>
       </c>
@@ -2035,16 +2151,20 @@
         <v>2</v>
       </c>
       <c r="C42" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D42" t="s">
-        <v>52</v>
-      </c>
-      <c r="E42" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E42" s="2">
+        <v>45202</v>
+      </c>
+      <c r="F42" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>3782468</v>
       </c>
@@ -2052,16 +2172,20 @@
         <v>5</v>
       </c>
       <c r="C43" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="D43" t="s">
-        <v>2</v>
-      </c>
-      <c r="E43" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E43" s="2">
+        <v>45202</v>
+      </c>
+      <c r="F43" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>3895904</v>
       </c>
@@ -2069,16 +2193,20 @@
         <v>3</v>
       </c>
       <c r="C44" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="D44" t="s">
-        <v>69</v>
-      </c>
-      <c r="E44" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E44" s="2">
+        <v>45202</v>
+      </c>
+      <c r="F44" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>4228740</v>
       </c>
@@ -2086,16 +2214,20 @@
         <v>3</v>
       </c>
       <c r="C45" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="D45" t="s">
-        <v>2</v>
-      </c>
-      <c r="E45" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E45" s="2">
+        <v>45202</v>
+      </c>
+      <c r="F45" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>4276060</v>
       </c>
@@ -2103,33 +2235,41 @@
         <v>2</v>
       </c>
       <c r="C46" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="D46" t="s">
-        <v>2</v>
-      </c>
-      <c r="E46" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E46" s="2">
+        <v>45202</v>
+      </c>
+      <c r="F46" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47">
-        <v>4300360</v>
+        <v>4775040</v>
       </c>
       <c r="B47">
         <v>3</v>
       </c>
       <c r="C47" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="D47" t="s">
-        <v>5</v>
-      </c>
-      <c r="E47" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E47" s="2">
+        <v>45202</v>
+      </c>
+      <c r="F47" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>4775040</v>
       </c>
@@ -2137,16 +2277,20 @@
         <v>2</v>
       </c>
       <c r="C48" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="D48" t="s">
-        <v>63</v>
-      </c>
-      <c r="E48" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E48" s="2">
+        <v>45202</v>
+      </c>
+      <c r="F48" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>3625575</v>
       </c>
@@ -2154,16 +2298,20 @@
         <v>2</v>
       </c>
       <c r="C49" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="D49" t="s">
-        <v>3</v>
-      </c>
-      <c r="E49" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E49" s="2">
+        <v>45203</v>
+      </c>
+      <c r="F49" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 15 dias</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>4651235</v>
       </c>
@@ -2171,16 +2319,20 @@
         <v>2</v>
       </c>
       <c r="C50" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="D50" t="s">
-        <v>2</v>
-      </c>
-      <c r="E50" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E50" s="2">
+        <v>45212</v>
+      </c>
+      <c r="F50" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 6 dias</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>3817415</v>
       </c>
@@ -2188,16 +2340,20 @@
         <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="D51" t="s">
-        <v>77</v>
-      </c>
-      <c r="E51" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="E51" s="2">
+        <v>45215</v>
+      </c>
+      <c r="F51" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 3 dias</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>4771389</v>
       </c>
@@ -2205,16 +2361,20 @@
         <v>2</v>
       </c>
       <c r="C52" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="D52" t="s">
-        <v>2</v>
-      </c>
-      <c r="E52" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E52" s="2">
+        <v>45215</v>
+      </c>
+      <c r="F52" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 8 meses e 3 dias</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>3417212</v>
       </c>
@@ -2222,16 +2382,20 @@
         <v>3</v>
       </c>
       <c r="C53" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D53" t="s">
-        <v>52</v>
-      </c>
-      <c r="E53" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E53" s="2">
+        <v>45230</v>
+      </c>
+      <c r="F53" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 7 meses e 19 dias</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>4222350</v>
       </c>
@@ -2239,16 +2403,20 @@
         <v>2</v>
       </c>
       <c r="C54" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="D54" t="s">
-        <v>81</v>
-      </c>
-      <c r="E54" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E54" s="2">
+        <v>45233</v>
+      </c>
+      <c r="F54" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 7 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>4298110</v>
       </c>
@@ -2256,16 +2424,20 @@
         <v>2</v>
       </c>
       <c r="C55" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="D55" t="s">
-        <v>83</v>
-      </c>
-      <c r="E55" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E55" s="2">
+        <v>45233</v>
+      </c>
+      <c r="F55" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 7 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>4276450</v>
       </c>
@@ -2273,16 +2445,20 @@
         <v>2</v>
       </c>
       <c r="C56" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="D56" t="s">
-        <v>85</v>
-      </c>
-      <c r="E56" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E56" s="2">
+        <v>45236</v>
+      </c>
+      <c r="F56" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 7 meses e 13 dias</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>3394972</v>
       </c>
@@ -2290,16 +2466,20 @@
         <v>2</v>
       </c>
       <c r="C57" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="D57" t="s">
-        <v>87</v>
-      </c>
-      <c r="E57" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E57" s="2">
+        <v>45243</v>
+      </c>
+      <c r="F57" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 7 meses e 6 dias</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>4200420</v>
       </c>
@@ -2307,16 +2487,20 @@
         <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="D58" t="s">
-        <v>77</v>
-      </c>
-      <c r="E58" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E58" s="2">
+        <v>45244</v>
+      </c>
+      <c r="F58" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 7 meses e 5 dias</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>4255798</v>
       </c>
@@ -2324,16 +2508,20 @@
         <v>4</v>
       </c>
       <c r="C59" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D59" t="s">
-        <v>2</v>
-      </c>
-      <c r="E59" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E59" s="2">
+        <v>45373</v>
+      </c>
+      <c r="F59" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 2 meses e 28 dias</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>3393801</v>
       </c>
@@ -2341,16 +2529,20 @@
         <v>2</v>
       </c>
       <c r="C60" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D60" t="s">
-        <v>2</v>
-      </c>
-      <c r="E60" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E60" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F60" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>3405206</v>
       </c>
@@ -2358,16 +2550,20 @@
         <v>3</v>
       </c>
       <c r="C61" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="D61" t="s">
-        <v>5</v>
-      </c>
-      <c r="E61" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="E61" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F61" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>3406539</v>
       </c>
@@ -2375,16 +2571,20 @@
         <v>2</v>
       </c>
       <c r="C62" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="D62" t="s">
-        <v>2</v>
-      </c>
-      <c r="E62" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E62" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F62" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>3409708</v>
       </c>
@@ -2392,16 +2592,20 @@
         <v>3</v>
       </c>
       <c r="C63" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="D63" t="s">
-        <v>94</v>
-      </c>
-      <c r="E63" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+      <c r="E63" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F63" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>3410943</v>
       </c>
@@ -2409,16 +2613,20 @@
         <v>3</v>
       </c>
       <c r="C64" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="D64" t="s">
         <v>2</v>
       </c>
-      <c r="E64" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E64" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F64" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>3411656</v>
       </c>
@@ -2426,16 +2634,20 @@
         <v>3</v>
       </c>
       <c r="C65" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="D65" t="s">
-        <v>2</v>
-      </c>
-      <c r="E65" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+      <c r="E65" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F65" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>3412547</v>
       </c>
@@ -2443,16 +2655,20 @@
         <v>4</v>
       </c>
       <c r="C66" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="D66" t="s">
-        <v>5</v>
-      </c>
-      <c r="E66" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="E66" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F66" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>3415260</v>
       </c>
@@ -2460,16 +2676,20 @@
         <v>3</v>
       </c>
       <c r="C67" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="D67" t="s">
-        <v>2</v>
-      </c>
-      <c r="E67" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E67" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F67" s="3" t="str">
+        <f t="shared" ref="F67:F95" ca="1" si="1">DATEDIF(E67,TODAY(),"y")&amp;" anos, "&amp;DATEDIF(E67,TODAY(),"ym")&amp;" meses e "&amp;DATEDIF(E67,TODAY(),"md")&amp;" dias"</f>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>3781755</v>
       </c>
@@ -2477,16 +2697,20 @@
         <v>2</v>
       </c>
       <c r="C68" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D68" t="s">
-        <v>2</v>
-      </c>
-      <c r="E68" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="E68" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F68" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>3866270</v>
       </c>
@@ -2494,16 +2718,20 @@
         <v>2</v>
       </c>
       <c r="C69" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="D69" t="s">
-        <v>2</v>
-      </c>
-      <c r="E69" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E69" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F69" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>3871479</v>
       </c>
@@ -2511,16 +2739,20 @@
         <v>7</v>
       </c>
       <c r="C70" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="D70" t="s">
-        <v>2</v>
-      </c>
-      <c r="E70" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="E70" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F70" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>4208595</v>
       </c>
@@ -2528,16 +2760,20 @@
         <v>2</v>
       </c>
       <c r="C71" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="D71" t="s">
-        <v>5</v>
-      </c>
-      <c r="E71" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+      <c r="E71" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F71" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>4466390</v>
       </c>
@@ -2545,16 +2781,20 @@
         <v>3</v>
       </c>
       <c r="C72" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="D72" t="s">
-        <v>106</v>
-      </c>
-      <c r="E72" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E72" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F72" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>4545265</v>
       </c>
@@ -2562,16 +2802,20 @@
         <v>3</v>
       </c>
       <c r="C73" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="D73" t="s">
-        <v>108</v>
-      </c>
-      <c r="E73" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E73" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F73" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>4774426</v>
       </c>
@@ -2579,16 +2823,20 @@
         <v>2</v>
       </c>
       <c r="C74" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="D74" t="s">
-        <v>110</v>
-      </c>
-      <c r="E74" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="E74" s="2">
+        <v>45377</v>
+      </c>
+      <c r="F74" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 24 dias</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>3405940</v>
       </c>
@@ -2596,16 +2844,20 @@
         <v>6</v>
       </c>
       <c r="C75" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="D75" t="s">
-        <v>2</v>
-      </c>
-      <c r="E75" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="E75" s="2">
+        <v>45378</v>
+      </c>
+      <c r="F75" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 23 dias</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>4958616</v>
       </c>
@@ -2613,16 +2865,20 @@
         <v>1</v>
       </c>
       <c r="C76" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="D76" t="s">
-        <v>2</v>
-      </c>
-      <c r="E76" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+      <c r="E76" s="2">
+        <v>45383</v>
+      </c>
+      <c r="F76" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 18 dias</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>4455959</v>
       </c>
@@ -2630,16 +2886,20 @@
         <v>2</v>
       </c>
       <c r="C77" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="D77" t="s">
-        <v>114</v>
-      </c>
-      <c r="E77" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+      <c r="E77" s="2">
+        <v>45384</v>
+      </c>
+      <c r="F77" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 17 dias</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>4772326</v>
       </c>
@@ -2647,16 +2907,20 @@
         <v>2</v>
       </c>
       <c r="C78" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="D78" t="s">
-        <v>2</v>
-      </c>
-      <c r="E78" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="E78" s="2">
+        <v>45385</v>
+      </c>
+      <c r="F78" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 16 dias</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>3634779</v>
       </c>
@@ -2664,16 +2928,20 @@
         <v>2</v>
       </c>
       <c r="C79" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="D79" t="s">
-        <v>118</v>
-      </c>
-      <c r="E79" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+        <v>103</v>
+      </c>
+      <c r="E79" s="2">
+        <v>45394</v>
+      </c>
+      <c r="F79" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 7 dias</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>3402592</v>
       </c>
@@ -2681,16 +2949,20 @@
         <v>5</v>
       </c>
       <c r="C80" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="D80" t="s">
-        <v>2</v>
-      </c>
-      <c r="E80" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+      <c r="E80" s="2">
+        <v>45399</v>
+      </c>
+      <c r="F80" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>3410889</v>
       </c>
@@ -2698,16 +2970,20 @@
         <v>2</v>
       </c>
       <c r="C81" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="D81" t="s">
-        <v>52</v>
-      </c>
-      <c r="E81" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+      <c r="E81" s="2">
+        <v>45399</v>
+      </c>
+      <c r="F81" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>3744418</v>
       </c>
@@ -2715,16 +2991,20 @@
         <v>2</v>
       </c>
       <c r="C82" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="D82" t="s">
-        <v>69</v>
-      </c>
-      <c r="E82" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+        <v>103</v>
+      </c>
+      <c r="E82" s="2">
+        <v>45399</v>
+      </c>
+      <c r="F82" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>3792056</v>
       </c>
@@ -2732,16 +3012,20 @@
         <v>2</v>
       </c>
       <c r="C83" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="D83" t="s">
-        <v>5</v>
-      </c>
-      <c r="E83" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="E83" s="2">
+        <v>45399</v>
+      </c>
+      <c r="F83" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>4207270</v>
       </c>
@@ -2749,16 +3033,20 @@
         <v>2</v>
       </c>
       <c r="C84" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="D84" t="s">
-        <v>52</v>
-      </c>
-      <c r="E84" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+      <c r="E84" s="2">
+        <v>45399</v>
+      </c>
+      <c r="F84" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>4223047</v>
       </c>
@@ -2766,16 +3054,20 @@
         <v>2</v>
       </c>
       <c r="C85" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="D85" t="s">
-        <v>5</v>
-      </c>
-      <c r="E85" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+        <v>103</v>
+      </c>
+      <c r="E85" s="2">
+        <v>45399</v>
+      </c>
+      <c r="F85" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>4285573</v>
       </c>
@@ -2783,16 +3075,20 @@
         <v>2</v>
       </c>
       <c r="C86" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="D86" t="s">
-        <v>5</v>
-      </c>
-      <c r="E86" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E86" s="2">
+        <v>45399</v>
+      </c>
+      <c r="F86" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 2 dias</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>3340732</v>
       </c>
@@ -2800,16 +3096,20 @@
         <v>2</v>
       </c>
       <c r="C87" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="D87" t="s">
-        <v>5</v>
-      </c>
-      <c r="E87" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+      <c r="E87" s="2">
+        <v>45400</v>
+      </c>
+      <c r="F87" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 1 dias</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>3386384</v>
       </c>
@@ -2817,16 +3117,20 @@
         <v>2</v>
       </c>
       <c r="C88" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="D88" t="s">
-        <v>2</v>
-      </c>
-      <c r="E88" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="E88" s="2">
+        <v>45400</v>
+      </c>
+      <c r="F88" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 1 dias</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>3408779</v>
       </c>
@@ -2834,16 +3138,20 @@
         <v>2</v>
       </c>
       <c r="C89" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="D89" t="s">
-        <v>2</v>
-      </c>
-      <c r="E89" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+      <c r="E89" s="2">
+        <v>45400</v>
+      </c>
+      <c r="F89" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 1 dias</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>3500837</v>
       </c>
@@ -2851,16 +3159,20 @@
         <v>3</v>
       </c>
       <c r="C90" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="D90" t="s">
-        <v>2</v>
-      </c>
-      <c r="E90" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="E90" s="2">
+        <v>45400</v>
+      </c>
+      <c r="F90" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 1 dias</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>3969789</v>
       </c>
@@ -2868,16 +3180,20 @@
         <v>2</v>
       </c>
       <c r="C91" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="D91" t="s">
-        <v>7</v>
-      </c>
-      <c r="E91" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="E91" s="2">
+        <v>45400</v>
+      </c>
+      <c r="F91" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 1 dias</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>4500202</v>
       </c>
@@ -2885,16 +3201,20 @@
         <v>2</v>
       </c>
       <c r="C92" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="D92" t="s">
-        <v>2</v>
-      </c>
-      <c r="E92" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="E92" s="2">
+        <v>45400</v>
+      </c>
+      <c r="F92" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 1 dias</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>3414620</v>
       </c>
@@ -2902,16 +3222,20 @@
         <v>4</v>
       </c>
       <c r="C93" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="D93" t="s">
-        <v>5</v>
-      </c>
-      <c r="E93" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="E93" s="2">
+        <v>45401</v>
+      </c>
+      <c r="F93" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 2 meses e 0 dias</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>4815866</v>
       </c>
@@ -2919,13 +3243,38 @@
         <v>2</v>
       </c>
       <c r="C94" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="D94" t="s">
-        <v>2</v>
-      </c>
-      <c r="E94" t="s">
-        <v>126</v>
+        <v>110</v>
+      </c>
+      <c r="E94" s="2">
+        <v>45404</v>
+      </c>
+      <c r="F94" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 1 meses e 28 dias</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" s="4">
+        <v>4775562</v>
+      </c>
+      <c r="B95" s="4">
+        <v>2</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E95" s="5">
+        <v>45097</v>
+      </c>
+      <c r="F95" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2 anos, 11 meses e 30 dias</v>
       </c>
     </row>
   </sheetData>

</xml_diff>